<commit_message>
R03 (em andamento): preço do gás das 4 distribuidoras (CVM), MIP v02 e variantes, quadro v02, prévia, executor de cenários e testes T9–T11
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CWPuQS1EQNnCbSqHfPPCuA
</commit_message>
<xml_diff>
--- a/parametros/quadro_parametros_v02.xlsx
+++ b/parametros/quadro_parametros_v02.xlsx
@@ -1143,10 +1143,10 @@
         <v>103034.3882686664</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>4152.654537533038</v>
+        <v>5771.092442464354</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.04030357832284907</v>
+        <v>0.05601132339832011</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1169,10 +1169,10 @@
         <v>590.7983845967136</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>128.429406067658</v>
+        <v>178.4829361672732</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.2173827982879904</v>
+        <v>0.3021046448681606</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1195,10 +1195,10 @@
         <v>1464.067669526863</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>318.2631268847263</v>
+        <v>442.3016433653686</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.2173827982879904</v>
+        <v>0.3021046448681607</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1221,10 +1221,10 @@
         <v>424.6040878846963</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>92.30162478889508</v>
+        <v>128.2748671799755</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.2173827982879904</v>
+        <v>0.3021046448681607</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1247,10 +1247,10 @@
         <v>1541.587401793107</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>455.799803067663</v>
+        <v>633.4412783402894</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.29566912815809</v>
+        <v>0.4109019557395826</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1273,10 +1273,10 @@
         <v>49.34845748188254</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>14.59081539961478</v>
+        <v>20.27737769203718</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.29566912815809</v>
+        <v>0.4109019557395827</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1299,10 +1299,10 @@
         <v>2876.45470183467</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>850.4788538776957</v>
+        <v>1181.940862580184</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.29566912815809</v>
+        <v>0.4109019557395827</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1325,10 +1325,10 @@
         <v>662.6289189346137</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>195.9189147537349</v>
+        <v>272.2755187198381</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.29566912815809</v>
+        <v>0.4109019557395827</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1351,10 +1351,10 @@
         <v>22.58659150614427</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>5.714851026378176</v>
+        <v>7.942132741851839</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1377,10 +1377,10 @@
         <v>1259.051543108248</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>377.0970518604561</v>
+        <v>524.0652518522081</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.2995088278352039</v>
+        <v>0.4162381236263265</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1403,10 +1403,10 @@
         <v>217.967061073277</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>55.14994515008586</v>
+        <v>76.6438500437028</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1429,10 +1429,10 @@
         <v>157.9716449979387</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>39.96992717159351</v>
+        <v>55.54763646746012</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
         <v>851.7982201766725</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>215.5216705238388</v>
+        <v>299.5181690905399</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1481,10 +1481,10 @@
         <v>1965.443268170884</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1590.118923887173</v>
+        <v>2209.845105419345</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.8090383221119368</v>
+        <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1507,10 +1507,10 @@
         <v>119.8337944186895</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>30.3203023281376</v>
+        <v>42.13720790824564</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1533,10 +1533,10 @@
         <v>3953.557802713218</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>3038.80198526845</v>
+        <v>4223.131737259013</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.7686246507343344</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>647.2898547259196</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>497.522938512588</v>
+        <v>691.4254110115246</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.7686246507343345</v>
+        <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1585,10 +1585,10 @@
         <v>200.8954216112138</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>154.4131732700461</v>
+        <v>214.593506207019</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.7686246507343346</v>
+        <v>1</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1611,10 +1611,10 @@
         <v>286.7236488018115</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>220.3828644175664</v>
+        <v>306.2739440021971</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.7686246507343345</v>
+        <v>1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1637,10 +1637,10 @@
         <v>1928.905902166182</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>488.0510577163718</v>
+        <v>678.2619997080068</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1663,10 +1663,10 @@
         <v>3322.234178981784</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>2177.597430699141</v>
+        <v>3026.284985050389</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.6554617505520162</v>
+        <v>0.9109186234360821</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1689,10 +1689,10 @@
         <v>2738.993933673587</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>2096.316438898289</v>
+        <v>2913.325885453203</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.7653600152690634</v>
+        <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1715,10 +1715,10 @@
         <v>2652.608321579856</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>704.9304407989232</v>
+        <v>979.6670304711964</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.265749916813605</v>
+        <v>0.3693221583078352</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1741,10 +1741,10 @@
         <v>1122.233344512993</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>283.9470656287933</v>
+        <v>394.6113864515563</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1767,10 +1767,10 @@
         <v>158.4584978450351</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>40.09311049884177</v>
+        <v>55.71882874037727</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1793,10 +1793,10 @@
         <v>557.1254084888648</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>140.963664732584</v>
+        <v>195.90224345596</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1819,10 +1819,10 @@
         <v>470.9133141670703</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>119.1503125237263</v>
+        <v>165.5874481992042</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1845,10 +1845,10 @@
         <v>548.1170452752175</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>138.684372005149</v>
+        <v>192.7346288820594</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1871,10 +1871,10 @@
         <v>1154.016557351937</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>291.9888423822634</v>
+        <v>405.7873310495164</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1897,10 +1897,10 @@
         <v>205.2552396080408</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>51.93360478602611</v>
+        <v>72.17398687554113</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268969</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1923,10 +1923,10 @@
         <v>316.4324450498808</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>80.06362017397512</v>
+        <v>111.2672747338276</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268969</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1949,10 +1949,10 @@
         <v>270.1399628646077</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>68.35071345858452</v>
+        <v>94.98942960765018</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1975,10 +1975,10 @@
         <v>4224.112165769647</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>15.2811455393217</v>
+        <v>21.23675416221056</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.003617599377013093</v>
+        <v>0.005027507160984954</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2001,10 +2001,10 @@
         <v>1704.94850383175</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>6.497797206130856</v>
+        <v>9.030221033326066</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2027,10 +2027,10 @@
         <v>21420.71414201967</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>81.6373375456967</v>
+        <v>113.4543260159486</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2053,10 +2053,10 @@
         <v>1496.336706942969</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>50.01190370456322</v>
+        <v>69.5033301937324</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.03342289437431368</v>
+        <v>0.04644899097324719</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2079,10 +2079,10 @@
         <v>1274.303775276272</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>4.856549914641455</v>
+        <v>6.749321007927743</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2105,10 +2105,10 @@
         <v>1597.079682805128</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>6.086694042416427</v>
+        <v>8.45889627232272</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2131,10 +2131,10 @@
         <v>2245.708314328186</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>8.55870847584645</v>
+        <v>11.89434308965078</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2157,10 +2157,10 @@
         <v>117.2355772354733</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.4468011816824767</v>
+        <v>0.6209355725563697</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2183,10 +2183,10 @@
         <v>436.1310913128293</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>1.662156587293009</v>
+        <v>2.309958421154293</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2209,10 +2209,10 @@
         <v>1884.74657169748</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>7.183032789739402</v>
+        <v>9.982517416790753</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2235,10 +2235,10 @@
         <v>894.8737012347408</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>3.410488834504348</v>
+        <v>4.73967823714267</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2261,10 +2261,10 @@
         <v>2338.444956025624</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>8.912140787715874</v>
+        <v>12.38552060646971</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2287,10 +2287,10 @@
         <v>914.612407881436</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>3.485715806235917</v>
+        <v>4.844223848655891</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2313,10 +2313,10 @@
         <v>1439.29117329178</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>5.485339963996378</v>
+        <v>7.623173014862262</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2339,10 +2339,10 @@
         <v>343.2675634889163</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>1.308240694649003</v>
+        <v>1.818108854847912</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2365,10 +2365,10 @@
         <v>301.5927543875164</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>1.149412168428696</v>
+        <v>1.597379174824421</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2391,10 +2391,10 @@
         <v>221.0196732403219</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.842336887039869</v>
+        <v>1.170625680240819</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2417,10 +2417,10 @@
         <v>8003.795783121474</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>30.50358515880481</v>
+        <v>42.39192260924876</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2443,10 +2443,10 @@
         <v>114.0627600051552</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0.4347091314602025</v>
+        <v>0.6041308181466463</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2469,10 +2469,10 @@
         <v>5756.222934834066</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>20.82370850300419</v>
+        <v>28.9394520251041</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.003617599377013092</v>
+        <v>0.005027507160984955</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2495,10 +2495,10 @@
         <v>1954.825572054542</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>7.071775771633773</v>
+        <v>9.82789956198072</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.003617599377013093</v>
+        <v>0.005027507160984955</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2521,10 +2521,10 @@
         <v>2690.879626450015</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>10.25531860902868</v>
+        <v>14.25218283502799</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2547,10 +2547,10 @@
         <v>1345.342038519903</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>4.866908520419125</v>
+        <v>6.76371673263291</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.003617599377013092</v>
+        <v>0.005027507160984955</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2573,10 +2573,10 @@
         <v>1823.681264435676</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>6.950304363030023</v>
+        <v>9.659086403594308</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2599,10 +2599,10 @@
         <v>1335.916829286847</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>5.091365880819523</v>
+        <v>7.075653149340416</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2625,10 +2625,10 @@
         <v>3335.111298113421</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>12.71057561346462</v>
+        <v>17.66434125430878</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -4155,11 +4155,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
@@ -5560,6 +5560,474 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>comgas_receita_liquida_gas_nao_termica_2019</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>8636.219999999999</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>R$ mi</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Comgás (Companhia de Gás de São Paulo) — DFP 31/12/2019 (CVM, Rede de Divulgação Externa)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Demonstrações Financeiras Padronizadas 2019</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Relatório da Administração, item 2, linha "Vendas de Gás" (PDF p. 14); = soma das receitas líquidas dos 5 segmentos da nota 5 (p. 27)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENETCONSULTA/frmDownloadDocumento.aspx?CodigoInstituicao=1&amp;NumeroSequencialDocumento=90958</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>dados/externos/brutos/gas/cvm_rad_comgas_dfp2019/comgas_dfp2019_v2.zip (fora do git)</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>d43e27aeb42cebf1b7dbf47925fdceb67c5e91cf157d087a6137f64ed5029bb3</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-10-15T19:43:01Z</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Receita líquida de venda de gás, sem construção (813.341 R$ mil) e sem prestação de serviços (64.660); não há segmento termelétrico na DFP (volume "ex-termo"). Extraído e conferido por verificadores céticos independentes (Rodada 03; workflow r03-cvm-preco-gas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>comgas_volume_nao_termico_2019</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>4512.371</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>milhões m³</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Comgás (Companhia de Gás de São Paulo) — DFP 31/12/2019 (CVM, Rede de Divulgação Externa)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Demonstrações Financeiras Padronizadas 2019</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Relatório da Administração (p. 14) e nota 5 (p. 27), "Volume ex-termo" = 279.450 + 160.573 + 3.516.469 + 333.800 + 222.079 mil m³</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENETCONSULTA/frmDownloadDocumento.aspx?CodigoInstituicao=1&amp;NumeroSequencialDocumento=90958</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>dados/externos/brutos/gas/cvm_rad_comgas_dfp2019/comgas_dfp2019_v2.zip (fora do git)</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>d43e27aeb42cebf1b7dbf47925fdceb67c5e91cf157d087a6137f64ed5029bb3</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-10-15T19:43:01Z</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Volumes dos mesmos 5 segmentos (residencial, comercial, industrial, cogeração, automotivo). O MME dá 14.239 milhões m³/d para a Comgás (inclui o térmico); a DFP dá 12.363. Extraído e conferido por verificadores céticos independentes (Rodada 03; workflow r03-cvm-preco-gas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ceg_receita_liquida_gas_nao_termica_2019</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>3573.676</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>R$ mi</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>CEG (Companhia Distribuidora de Gás do Rio de Janeiro) — DFP 31/12/2019 (CVM, Rede de Divulgação Externa)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Demonstrações Financeiras Padronizadas 2019</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Nota 22, "Margem por segmento em 2019" (PDF p. 99): residencial 729.958 + comercial 266.030 + industrial 823.790 + automotivo 1.753.898 R$ mil</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENETCONSULTA/frmDownloadDocumento.aspx?CodigoInstituicao=1&amp;NumeroSequencialDocumento=91986</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>dados/externos/brutos/gas/cvm_rad_ceg_dfp2019/ceg_dfp2019.zip (fora do git)</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>60aa81f4936c3af9dd1856c114b63cd5057039179a81902578b319efea815d57</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-10-15T19:44:19Z</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Receita líquida por segmento alocada pela companhia; fora: termelétrico (845.815), construção (102.662) e outras receitas (108.959). Extraído e conferido por verificadores céticos independentes (Rodada 03; workflow r03-cvm-preco-gas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ceg_volume_nao_termico_2019</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>1628.581</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>milhões m³</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CEG (Companhia Distribuidora de Gás do Rio de Janeiro) — DFP 31/12/2019 (CVM, Rede de Divulgação Externa)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Demonstrações Financeiras Padronizadas 2019</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Nota 22 (PDF p. 99): 112.699 + 73.742 + 434.927 + 1.007.213 mil m³ (= 2.792.598 − termelétrico 1.164.017)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENETCONSULTA/frmDownloadDocumento.aspx?CodigoInstituicao=1&amp;NumeroSequencialDocumento=91986</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>dados/externos/brutos/gas/cvm_rad_ceg_dfp2019/ceg_dfp2019.zip (fora do git)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>60aa81f4936c3af9dd1856c114b63cd5057039179a81902578b319efea815d57</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-10-15T19:44:19Z</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Volumes marcados como não auditados. Extraído e conferido por verificadores céticos independentes (Rodada 03; workflow r03-cvm-preco-gas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>gasmig_receita_liquida_gas_nao_termica_2019</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1638.357</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>R$ mi</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Gasmig (Companhia de Gás de Minas Gerais) — DFP 31/12/2019 (CVM, Rede de Divulgação Externa)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Demonstrações Financeiras Padronizadas 2019</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Nota 19 (PDF p. 93): receita líquida sem construção 1.815.078 R$ mil × (bruta não térmica 2.077.951 ÷ bruta total 2.302.089)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENETCONSULTA/frmDownloadDocumento.aspx?CodigoInstituicao=1&amp;NumeroSequencialDocumento=92390</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>dados/externos/brutos/gas/cvm_rad_gasmig_dfp2019/gasmig_dfp2019.zip (fora do git)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>a595910856fda5e8b4f5a6aa9d66c59de254e5df1721142549123e828d1208fa</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-10-15T19:45:02Z</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>APROXIMAÇÃO: a Gasmig não divulga deduções por segmento (nota 26: segmento único); deduções rateadas na proporção da receita bruta. Pior caso (térmico sem deduções): 1590.940. Extraído e conferido por verificadores céticos independentes (Rodada 03; workflow r03-cvm-preco-gas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>gasmig_volume_nao_termico_2019</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>839.864</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>milhões m³</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Gasmig (Companhia de Gás de Minas Gerais) — DFP 31/12/2019 (CVM, Rede de Divulgação Externa)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Demonstrações Financeiras Padronizadas 2019</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Nota 19 (PDF p. 93), "Subtotal - gás convencional" = RA (p. 43) "Total Mercado Não Térmico"</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENETCONSULTA/frmDownloadDocumento.aspx?CodigoInstituicao=1&amp;NumeroSequencialDocumento=92390</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>dados/externos/brutos/gas/cvm_rad_gasmig_dfp2019/gasmig_dfp2019.zip (fora do git)</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>a595910856fda5e8b4f5a6aa9d66c59de254e5df1721142549123e828d1208fa</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-10-15T19:45:02Z</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Volume total 1.129.653 mil m³; térmico 289.789. Extraído e conferido por verificadores céticos independentes (Rodada 03; workflow r03-cvm-preco-gas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>sulgas_receita_liquida_gas_sem_servico_2019</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>889.79883949</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>R$ mi</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Sulgás (CAGE/Sefaz-RS)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Demonstrações Contábeis Sulgás 2019, Nota 18</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>PDF p. 86: receita líquida total 898.710.338,54 − segmento Serviço 8.911.499,05</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>dados/externos/brutos/gas/cage_rs_2019/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf (fora do git)</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>94cf3c42af64318d52194bc03ff75a478f00268d97a4fc6a45a2a4ce71d58a5f</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-10-15T19:34:32Z</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Para o preço médio comparável às outras 3 distribuidoras (só venda de gás, sem serviço). Volume: 646.361921 milhões m³ (total − Serviço).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>gas_preco_medio_4_distribuidoras_2019</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>1.932307334658018</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>R$/m³</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>cálculo do projeto com as DFP 2019 de Sulgás, Comgás, CEG e Gasmig</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ver linhas sulgas_*, comgas_*, ceg_*, gasmig_*</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Σ receita líquida de venda de gás não térmica (14738.052 R$ mi) ÷ Σ volume não térmico (7627.178 milhões m³)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>não (calculado)</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>D9-b da Rodada 03: preço médio ponderado pelo volume. Com a receita total da Sulgás (898.71, com serviço): 1.933476. Só a Sulgás: 1.390413. A Gasmig é aproximação (deduções rateadas).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5571,7 +6039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -6893,20 +7361,20 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>VBP_GAS-RB (D9-b, usado)</t>
+          <t>preço médio ponderado das 4 distribuidoras (Sulgás, Comgás, CEG, Gasmig)</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>19421.04544377357</v>
+        <v>1.932307334658018</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>R$ mi</t>
+          <t>R$/m³</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>D9-b: preço da Sulgás 2019 (1.390413 R$/m³; Sulgás (demonstrações contábeis publicadas pela CAGE/Sefaz-RS), Prestação de Contas do Governador 2019, Volume V parte 2 (Setor Empresarial), Demonstrações Contábeis da Sulgás 2019, DRE (PDF p. 69, 'Receita líquida - venda de gás e serviços' (Nota 17), 31/12/2019 = 898.710.338,54; repetido na Nota 18 (p. 86)); acesso 2026-10-15T19:34:32Z; https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf) × volume não térmico do RB (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf); preço das 4 distribuidoras não reconferido</t>
+          <t>cálculo do projeto com as DFP 2019 de Sulgás, Comgás, CEG e Gasmig, ver linhas sulgas_*, comgas_*, ceg_*, gasmig_* (Σ receita líquida de venda de gás não térmica (14738.052 R$ mi) ÷ Σ volume não térmico (7627.178 milhões m³)); acesso 2026-10-16; nan</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -6914,21 +7382,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>VBP</t>
+          <t>gás</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>VBP da geração = E_r = F_r − T_r − G_r</t>
+          <t>VBP_GAS-RB (D9-b, usado)</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>4150.587165985572</v>
+        <v>26990.12103518296</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -6937,10 +7405,14 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>âncora por componentes (D3 = A)</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
+          <t>D9-b: preço médio das 4 distribuidoras (cálculo do projeto com as DFP 2019 de Sulgás, Comgás, CEG e Gasmig, ver linhas sulgas_*, comgas_*, ceg_*, gasmig_* (Σ receita líquida de venda de gás não térmica (14738.052 R$ mi) ÷ Σ volume não térmico (7627.178 milhões m³)); acesso 2026-10-16; nan) × volume não térmico (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>1.932307 × 13967.8200</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6955,11 +7427,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>VBP da distribuição = X_r − E_r − T_r − VBP_GAS</t>
+          <t>VBP da geração = E_r = F_r − T_r − G_r</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14384.2967767677</v>
+        <v>4150.587165985572</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -6968,7 +7440,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>resíduo (Seção 6.3 da Rodada 02)</t>
+          <t>âncora por componentes (D3 = A)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -6981,16 +7453,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>VBP da geração = E_r = F_r − T_r − G_r</t>
+          <t>VBP da distribuição = X_r − E_r − T_r − VBP_GAS</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>73164.04063037722</v>
+        <v>14384.2967767677</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -6999,7 +7471,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>âncora por componentes (D3 = A)</t>
+          <t>resíduo (Seção 6.3 da Rodada 02)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -7017,11 +7489,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>VBP da distribuição = X_r − E_r − T_r − VBP_GAS</t>
+          <t>VBP da geração = E_r = F_r − T_r − G_r</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>208427.8922088759</v>
+        <v>73164.04063037722</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7030,7 +7502,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>resíduo (Seção 6.3 da Rodada 02)</t>
+          <t>âncora por componentes (D3 = A)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -7038,30 +7510,30 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>gás por comprador (RS, D10)</t>
+          <t>VBP</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>participação: indústria + cogeração</t>
+          <t>VBP da distribuição = X_r − E_r − T_r − VBP_GAS</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.7649296324406342</v>
+        <v>200858.8166174665</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>fração</t>
+          <t>R$ mi</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Sulgás 2019, Nota 18 (receita líquida por segmento; dados/externos/gas/sulgas_segmentos_2019_v01.csv)</t>
+          <t>resíduo (Seção 6.3 da Rodada 02)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -7079,11 +7551,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>participação: automotivo</t>
+          <t>participação: indústria + cogeração</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.160005019930679</v>
+        <v>0.7649296324406342</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -7110,11 +7582,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>participação: residencial + comercial</t>
+          <t>participação: automotivo</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.06514947299384387</v>
+        <v>0.160005019930679</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -7141,11 +7613,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>participação: serviço</t>
+          <t>participação: residencial + comercial</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.009915874634843056</v>
+        <v>0.06514947299384387</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -7162,7 +7634,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CEMPRE</t>
+          <t>gás por comprador (RS, D10)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7172,13 +7644,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>composição remuneracoes</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>geracao 0.2365, S38_TRA 0.1075, S38_DIS 0.6234, S38_GAS 0.0326</t>
-        </is>
+          <t>participação: serviço</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0.009915874634843056</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -7187,7 +7657,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>IBGE, CEMPRE 2019 (SIDRA 6450); sigilosos do RS por diferença e proporção nacional; RB = Brasil − RS</t>
+          <t>Sulgás 2019, Nota 18 (receita líquida por segmento; dados/externos/gas/sulgas_segmentos_2019_v01.csv)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
@@ -7205,12 +7675,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>composição ocupacoes</t>
+          <t>composição remuneracoes</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>geracao 0.1772, S38_TRA 0.0563, S38_DIS 0.7374, S38_GAS 0.0290</t>
+          <t>geracao 0.2365, S38_TRA 0.1075, S38_DIS 0.6234, S38_GAS 0.0326</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -7233,17 +7703,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>composição remuneracoes</t>
+          <t>composição ocupacoes</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>geracao 0.4113, S38_TRA 0.1296, S38_DIS 0.4151, S38_GAS 0.0440</t>
+          <t>geracao 0.1772, S38_TRA 0.0563, S38_DIS 0.7374, S38_GAS 0.0290</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -7271,12 +7741,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>composição ocupacoes</t>
+          <t>composição remuneracoes</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>geracao 0.2970, S38_TRA 0.1212, S38_DIS 0.5426, S38_GAS 0.0391</t>
+          <t>geracao 0.4113, S38_TRA 0.1296, S38_DIS 0.4151, S38_GAS 0.0440</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -7294,30 +7764,32 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>CEMPRE</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>consumo específico S38_CAR</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>0.2414815886565868</v>
+          <t>composição ocupacoes</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>geracao 0.2970, S38_TRA 0.1212, S38_DIS 0.5426, S38_GAS 0.0391</t>
+        </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>tep/MWh</t>
+          <t>fração</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>EPE, BEN 2020, Tabela 5.4 – Centrais Elétricas de Serviço Público (p. 112); acesso 2026-10-15T19:38:26Z: consumo de combustível ÷ geração, por fonte</t>
+          <t>IBGE, CEMPRE 2019 (SIDRA 6450); sigilosos do RS por diferença e proporção nacional; RB = Brasil − RS</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -7335,11 +7807,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>consumo específico S38_GN</t>
+          <t>consumo específico S38_CAR</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.1971973023509885</v>
+        <v>0.2414815886565868</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -7366,11 +7838,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>consumo específico S38_PET</t>
+          <t>consumo específico S38_GN</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.2654644579576431</v>
+        <v>0.1971973023509885</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -7397,11 +7869,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>consumo específico S38_BIO</t>
+          <t>consumo específico S38_PET</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.2358695652173913</v>
+        <v>0.2654644579576431</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -7428,11 +7900,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>consumo específico S38_NUC</t>
+          <t>consumo específico S38_BIO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.2532705065410131</v>
+        <v>0.2358695652173913</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -7449,37 +7921,33 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>emissões</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>*</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>CO2e SEEG S38_CAR</t>
+          <t>consumo específico S38_NUC</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>3766364.701879445</v>
+        <v>0.2532705065410131</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>t CO2e</t>
+          <t>tep/MWh</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>SEEG 13.0, Dados nacionais, CO2e (t) GWP-AR5, 2019, Geração de eletricidade (serviço público); PET do RS (diesel + óleo, 17.8 mil t) realocado a CAR e GN ∝ GWh</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>fator E1 = 1.4347 t/MWh</t>
-        </is>
-      </c>
+          <t>EPE, BEN 2020, Tabela 5.4 – Centrais Elétricas de Serviço Público (p. 112); acesso 2026-10-15T19:38:26Z: consumo de combustível ÷ geração, por fonte</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7494,11 +7962,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CO2e SEEG S38_GN</t>
+          <t>CO2e SEEG S38_CAR</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>76185.42712055544</v>
+        <v>3766364.701879445</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -7512,7 +7980,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>fator E1 = 0.4364 t/MWh</t>
+          <t>fator E1 = 1.4347 t/MWh</t>
         </is>
       </c>
     </row>
@@ -7529,11 +7997,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CO2e SEEG S38_BIO</t>
+          <t>CO2e SEEG S38_GN</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>3.375718</v>
+        <v>76185.42712055544</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -7547,7 +8015,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>fator E1 = 0.0000 t/MWh</t>
+          <t>fator E1 = 0.4364 t/MWh</t>
         </is>
       </c>
     </row>
@@ -7559,16 +8027,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CO2e SEEG S38_CAR</t>
+          <t>CO2e SEEG S38_BIO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>9708245</v>
+        <v>3.375718</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -7577,12 +8045,12 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>SEEG 13.0, Dados nacionais, CO2e (t) GWP-AR5, 2019, Geração de eletricidade (serviço público); 'Não alocado' somado ao RB</t>
+          <t>SEEG 13.0, Dados nacionais, CO2e (t) GWP-AR5, 2019, Geração de eletricidade (serviço público); PET do RS (diesel + óleo, 17.8 mil t) realocado a CAR e GN ∝ GWh</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>fator E1 = 0.8670 t/MWh</t>
+          <t>fator E1 = 0.0000 t/MWh</t>
         </is>
       </c>
     </row>
@@ -7599,11 +8067,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CO2e SEEG S38_GN</t>
+          <t>CO2e SEEG S38_CAR</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>20513045.65</v>
+        <v>9708245</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -7617,7 +8085,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>fator E1 = 0.4326 t/MWh</t>
+          <t>fator E1 = 0.8670 t/MWh</t>
         </is>
       </c>
     </row>
@@ -7634,11 +8102,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CO2e SEEG S38_PET</t>
+          <t>CO2e SEEG S38_GN</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>4291625.8815</v>
+        <v>20513045.65</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -7652,7 +8120,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>fator E1 = 0.8295 t/MWh</t>
+          <t>fator E1 = 0.4326 t/MWh</t>
         </is>
       </c>
     </row>
@@ -7669,11 +8137,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CO2e SEEG S38_BIO</t>
+          <t>CO2e SEEG S38_PET</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>12196.055247059</v>
+        <v>4291625.8815</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -7687,40 +8155,44 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>fator E1 = 0.0069 t/MWh</t>
+          <t>fator E1 = 0.8295 t/MWh</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>emissões</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>κ (participação máxima do combustível na receita das térmicas)</t>
+          <t>CO2e SEEG S38_BIO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.7</v>
+        <v>12196.055247059</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>fração</t>
+          <t>t CO2e</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>HIPÓTESE das instruções da Rodada 03 (D9-f); variantes 0.60 e 0.80</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr"/>
+          <t>SEEG 13.0, Dados nacionais, CO2e (t) GWP-AR5, 2019, Geração de eletricidade (serviço público); 'Não alocado' somado ao RB</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>fator E1 = 0.0069 t/MWh</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7735,23 +8207,54 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
+          <t>κ (participação máxima do combustível na receita das térmicas)</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>fração</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>HIPÓTESE das instruções da Rodada 03 (D9-f); variantes 0.60 e 0.80</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
           <t>η (EOB mínimo ÷ VBP)</t>
         </is>
       </c>
-      <c r="D68" t="n">
+      <c r="D69" t="n">
         <v>0.1</v>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>fração</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>HIPÓTESE das instruções da Rodada 03 (D9-r); variante 0.05</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8827,11 +9330,11 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>19421.04544377357</v>
+        <v>26990.12103518296</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>D9-b: preço da Sulgás 2019 (1.390413 R$/m³; Sulgás (demonstrações contábeis publicadas pela CAGE/Sefaz-RS), Prestação de Contas do Governador 2019, Volume V parte 2 (Setor Empresarial), Demonstrações Contábeis da Sulgás 2019, DRE (PDF p. 69, 'Receita líquida - venda de gás e serviços' (Nota 17), 31/12/2019 = 898.710.338,54; repetido na Nota 18 (p. 86)); acesso 2026-10-15T19:34:32Z; https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf) × volume não térmico do RB (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf); preço das 4 distribuidoras não reconferido</t>
+          <t>D9-b: preço médio das 4 distribuidoras (cálculo do projeto com as DFP 2019 de Sulgás, Comgás, CEG e Gasmig, ver linhas sulgas_*, comgas_*, ceg_*, gasmig_* (Σ receita líquida de venda de gás não térmica (14738.052 R$ mi) ÷ Σ volume não térmico (7627.178 milhões m³)); acesso 2026-10-16; nan) × volume não térmico (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
         </is>
       </c>
     </row>
@@ -9454,7 +9957,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.04030357832284907</v>
+        <v>0.05601132339832011</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -9463,7 +9966,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4152.6545 ÷ compras ao S38 103034.3883; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 5771.0924 ÷ compras ao S38 103034.3883; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9494,7 +9997,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.959696421677151</v>
+        <v>0.9439886766016798</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -9503,7 +10006,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4152.6545 ÷ compras ao S38 103034.3883; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 5771.0924 ÷ compras ao S38 103034.3883; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9534,7 +10037,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.2173827982879904</v>
+        <v>0.3021046448681606</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -9543,7 +10046,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 128.4294 ÷ compras ao S38 590.7984; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 178.4829 ÷ compras ao S38 590.7984; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9574,7 +10077,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.7826172017120097</v>
+        <v>0.6978953551318394</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -9583,7 +10086,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 128.4294 ÷ compras ao S38 590.7984; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 178.4829 ÷ compras ao S38 590.7984; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9614,7 +10117,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.2173827982879904</v>
+        <v>0.3021046448681607</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -9623,7 +10126,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 318.2631 ÷ compras ao S38 1464.0677; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 442.3016 ÷ compras ao S38 1464.0677; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9654,7 +10157,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.7826172017120097</v>
+        <v>0.6978953551318393</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -9663,7 +10166,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 318.2631 ÷ compras ao S38 1464.0677; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 442.3016 ÷ compras ao S38 1464.0677; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9694,7 +10197,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.2173827982879904</v>
+        <v>0.3021046448681607</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -9703,7 +10206,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 92.3016 ÷ compras ao S38 424.6041; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 128.2749 ÷ compras ao S38 424.6041; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9734,7 +10237,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.7826172017120097</v>
+        <v>0.6978953551318393</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -9743,7 +10246,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 92.3016 ÷ compras ao S38 424.6041; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 128.2749 ÷ compras ao S38 424.6041; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9774,7 +10277,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.29566912815809</v>
+        <v>0.4109019557395826</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -9783,7 +10286,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 455.7998 ÷ compras ao S38 1541.5874; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 633.4413 ÷ compras ao S38 1541.5874; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9814,7 +10317,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.70433087184191</v>
+        <v>0.5890980442604175</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -9823,7 +10326,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 455.7998 ÷ compras ao S38 1541.5874; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 633.4413 ÷ compras ao S38 1541.5874; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9854,7 +10357,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.29566912815809</v>
+        <v>0.4109019557395827</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -9863,7 +10366,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 14.5908 ÷ compras ao S38 49.3485; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 20.2774 ÷ compras ao S38 49.3485; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9894,7 +10397,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.70433087184191</v>
+        <v>0.5890980442604173</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -9903,7 +10406,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 14.5908 ÷ compras ao S38 49.3485; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 20.2774 ÷ compras ao S38 49.3485; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9934,7 +10437,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.29566912815809</v>
+        <v>0.4109019557395827</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -9943,7 +10446,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 850.4789 ÷ compras ao S38 2876.4547; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1181.9409 ÷ compras ao S38 2876.4547; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -9974,7 +10477,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.7043308718419099</v>
+        <v>0.5890980442604173</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -9983,7 +10486,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 850.4789 ÷ compras ao S38 2876.4547; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1181.9409 ÷ compras ao S38 2876.4547; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10014,7 +10517,7 @@
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0.29566912815809</v>
+        <v>0.4109019557395827</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -10023,7 +10526,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 195.9189 ÷ compras ao S38 662.6289; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 272.2755 ÷ compras ao S38 662.6289; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10557,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.70433087184191</v>
+        <v>0.5890980442604173</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -10063,7 +10566,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 195.9189 ÷ compras ao S38 662.6289; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 272.2755 ÷ compras ao S38 662.6289; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10094,7 +10597,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -10103,7 +10606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 5.7149 ÷ compras ao S38 22.5866; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.9421 ÷ compras ao S38 22.5866; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10134,7 +10637,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.746980369976428</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -10143,7 +10646,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 5.7149 ÷ compras ao S38 22.5866; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.9421 ÷ compras ao S38 22.5866; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10174,7 +10677,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.2995088278352039</v>
+        <v>0.4162381236263265</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -10183,7 +10686,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 377.0971 ÷ compras ao S38 1259.0515; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 524.0653 ÷ compras ao S38 1259.0515; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10717,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.7004911721647962</v>
+        <v>0.5837618763736735</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -10223,7 +10726,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 377.0971 ÷ compras ao S38 1259.0515; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 524.0653 ÷ compras ao S38 1259.0515; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10757,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -10263,7 +10766,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 55.1499 ÷ compras ao S38 217.9671; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 76.6439 ÷ compras ao S38 217.9671; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10294,7 +10797,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.746980369976428</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -10303,7 +10806,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 55.1499 ÷ compras ao S38 217.9671; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 76.6439 ÷ compras ao S38 217.9671; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10334,7 +10837,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -10343,7 +10846,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 39.9699 ÷ compras ao S38 157.9716; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 55.5476 ÷ compras ao S38 157.9716; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10374,7 +10877,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -10383,7 +10886,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 39.9699 ÷ compras ao S38 157.9716; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 55.5476 ÷ compras ao S38 157.9716; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10414,7 +10917,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -10423,7 +10926,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 215.5217 ÷ compras ao S38 851.7982; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 299.5182 ÷ compras ao S38 851.7982; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10454,7 +10957,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.746980369976428</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -10463,7 +10966,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 215.5217 ÷ compras ao S38 851.7982; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 299.5182 ÷ compras ao S38 851.7982; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10494,7 +10997,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.8090383221119368</v>
+        <v>1</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -10503,7 +11006,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1590.1189 ÷ compras ao S38 1965.4433; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2209.8451 ÷ compras ao S38 1965.4433 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10534,7 +11037,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.1909616778880632</v>
+        <v>0</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -10543,7 +11046,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1590.1189 ÷ compras ao S38 1965.4433; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2209.8451 ÷ compras ao S38 1965.4433 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10574,7 +11077,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -10583,7 +11086,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 30.3203 ÷ compras ao S38 119.8338; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 42.1372 ÷ compras ao S38 119.8338; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10614,7 +11117,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -10623,7 +11126,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 30.3203 ÷ compras ao S38 119.8338; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 42.1372 ÷ compras ao S38 119.8338; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10654,7 +11157,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.7686246507343344</v>
+        <v>1</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -10663,7 +11166,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 3038.8020 ÷ compras ao S38 3953.5578; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4223.1317 ÷ compras ao S38 3953.5578 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10694,7 +11197,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.2313753492656656</v>
+        <v>0</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -10703,7 +11206,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 3038.8020 ÷ compras ao S38 3953.5578; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4223.1317 ÷ compras ao S38 3953.5578 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10734,7 +11237,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.7686246507343345</v>
+        <v>1</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -10743,7 +11246,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 497.5229 ÷ compras ao S38 647.2899; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 691.4254 ÷ compras ao S38 647.2899 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10774,7 +11277,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.2313753492656655</v>
+        <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -10783,7 +11286,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 497.5229 ÷ compras ao S38 647.2899; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 691.4254 ÷ compras ao S38 647.2899 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10814,7 +11317,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.7686246507343346</v>
+        <v>1</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -10823,7 +11326,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 154.4132 ÷ compras ao S38 200.8954; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 214.5935 ÷ compras ao S38 200.8954 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10854,7 +11357,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.2313753492656654</v>
+        <v>0</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -10863,7 +11366,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 154.4132 ÷ compras ao S38 200.8954; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 214.5935 ÷ compras ao S38 200.8954 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10894,7 +11397,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.7686246507343345</v>
+        <v>1</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -10903,7 +11406,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 220.3829 ÷ compras ao S38 286.7236; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 306.2739 ÷ compras ao S38 286.7236 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10934,7 +11437,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.2313753492656655</v>
+        <v>0</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -10943,7 +11446,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 220.3829 ÷ compras ao S38 286.7236; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 306.2739 ÷ compras ao S38 286.7236 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -10974,7 +11477,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -10983,7 +11486,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 488.0511 ÷ compras ao S38 1928.9059; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 678.2620 ÷ compras ao S38 1928.9059; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11014,7 +11517,7 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -11023,7 +11526,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 488.0511 ÷ compras ao S38 1928.9059; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 678.2620 ÷ compras ao S38 1928.9059; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11054,7 +11557,7 @@
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.6554617505520162</v>
+        <v>0.9109186234360821</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -11063,7 +11566,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2177.5974 ÷ compras ao S38 3322.2342; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 3026.2850 ÷ compras ao S38 3322.2342; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11094,7 +11597,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.3445382494479838</v>
+        <v>0.0890813765639179</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -11103,7 +11606,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2177.5974 ÷ compras ao S38 3322.2342; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 3026.2850 ÷ compras ao S38 3322.2342; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11134,7 +11637,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.7653600152690634</v>
+        <v>1</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -11143,7 +11646,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2096.3164 ÷ compras ao S38 2738.9939; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2913.3259 ÷ compras ao S38 2738.9939 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11174,7 +11677,7 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0.2346399847309366</v>
+        <v>0</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -11183,7 +11686,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2096.3164 ÷ compras ao S38 2738.9939; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2913.3259 ÷ compras ao S38 2738.9939 (limitado a 1); HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11214,7 +11717,7 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.265749916813605</v>
+        <v>0.3693221583078352</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -11223,7 +11726,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 704.9304 ÷ compras ao S38 2652.6083; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 979.6670 ÷ compras ao S38 2652.6083; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11254,7 +11757,7 @@
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.734250083186395</v>
+        <v>0.6306778416921648</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -11263,7 +11766,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 704.9304 ÷ compras ao S38 2652.6083; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 979.6670 ÷ compras ao S38 2652.6083; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11294,7 +11797,7 @@
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -11303,7 +11806,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 283.9471 ÷ compras ao S38 1122.2333; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 394.6114 ÷ compras ao S38 1122.2333; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11837,7 @@
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>0.746980369976428</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -11343,7 +11846,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 283.9471 ÷ compras ao S38 1122.2333; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 394.6114 ÷ compras ao S38 1122.2333; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11374,7 +11877,7 @@
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -11383,7 +11886,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 40.0931 ÷ compras ao S38 158.4585; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 55.7188 ÷ compras ao S38 158.4585; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11414,7 +11917,7 @@
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -11423,7 +11926,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 40.0931 ÷ compras ao S38 158.4585; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 55.7188 ÷ compras ao S38 158.4585; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11454,7 +11957,7 @@
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -11463,7 +11966,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 140.9637 ÷ compras ao S38 557.1254; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 195.9022 ÷ compras ao S38 557.1254; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11494,7 +11997,7 @@
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -11503,7 +12006,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 140.9637 ÷ compras ao S38 557.1254; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 195.9022 ÷ compras ao S38 557.1254; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11534,7 +12037,7 @@
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -11543,7 +12046,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 119.1503 ÷ compras ao S38 470.9133; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 165.5874 ÷ compras ao S38 470.9133; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11574,7 +12077,7 @@
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.746980369976428</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -11583,7 +12086,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 119.1503 ÷ compras ao S38 470.9133; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 165.5874 ÷ compras ao S38 470.9133; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11614,7 +12117,7 @@
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -11623,7 +12126,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 138.6844 ÷ compras ao S38 548.1170; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 192.7346 ÷ compras ao S38 548.1170; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11654,7 +12157,7 @@
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.746980369976428</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -11663,7 +12166,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 138.6844 ÷ compras ao S38 548.1170; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 192.7346 ÷ compras ao S38 548.1170; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11694,7 +12197,7 @@
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -11703,7 +12206,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 291.9888 ÷ compras ao S38 1154.0166; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 405.7873 ÷ compras ao S38 1154.0166; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11734,7 +12237,7 @@
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -11743,7 +12246,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 291.9888 ÷ compras ao S38 1154.0166; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 405.7873 ÷ compras ao S38 1154.0166; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11774,7 +12277,7 @@
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268969</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -11783,7 +12286,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 51.9336 ÷ compras ao S38 205.2552; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 72.1740 ÷ compras ao S38 205.2552; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11814,7 +12317,7 @@
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731031</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -11823,7 +12326,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 51.9336 ÷ compras ao S38 205.2552; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 72.1740 ÷ compras ao S38 205.2552; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11854,7 +12357,7 @@
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268969</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -11863,7 +12366,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 80.0636 ÷ compras ao S38 316.4324; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 111.2673 ÷ compras ao S38 316.4324; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11894,7 +12397,7 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731031</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -11903,7 +12406,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 80.0636 ÷ compras ao S38 316.4324; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 111.2673 ÷ compras ao S38 316.4324; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11934,7 +12437,7 @@
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.253019630023572</v>
+        <v>0.3516304237268968</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -11943,7 +12446,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 68.3507 ÷ compras ao S38 270.1400; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 94.9894 ÷ compras ao S38 270.1400; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -11974,7 +12477,7 @@
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.7469803699764279</v>
+        <v>0.6483695762731032</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -11983,7 +12486,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 68.3507 ÷ compras ao S38 270.1400; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 94.9894 ÷ compras ao S38 270.1400; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12014,7 +12517,7 @@
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.003617599377013093</v>
+        <v>0.005027507160984954</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -12023,7 +12526,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 15.2811 ÷ compras ao S38 4224.1122; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 21.2368 ÷ compras ao S38 4224.1122; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12054,7 +12557,7 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.9963824006229869</v>
+        <v>0.994972492839015</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -12063,7 +12566,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 15.2811 ÷ compras ao S38 4224.1122; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 21.2368 ÷ compras ao S38 4224.1122; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12094,7 +12597,7 @@
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -12103,7 +12606,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.4978 ÷ compras ao S38 1704.9485; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 9.0302 ÷ compras ao S38 1704.9485; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12134,7 +12637,7 @@
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -12143,7 +12646,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.4978 ÷ compras ao S38 1704.9485; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 9.0302 ÷ compras ao S38 1704.9485; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12174,7 +12677,7 @@
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -12183,7 +12686,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 81.6373 ÷ compras ao S38 21420.7141; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 113.4543 ÷ compras ao S38 21420.7141; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12214,7 +12717,7 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -12223,7 +12726,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 81.6373 ÷ compras ao S38 21420.7141; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 113.4543 ÷ compras ao S38 21420.7141; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12254,7 +12757,7 @@
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>0.03342289437431368</v>
+        <v>0.04644899097324719</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -12263,7 +12766,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 50.0119 ÷ compras ao S38 1496.3367; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 69.5033 ÷ compras ao S38 1496.3367; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12294,7 +12797,7 @@
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>0.9665771056256863</v>
+        <v>0.9535510090267528</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -12303,7 +12806,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 50.0119 ÷ compras ao S38 1496.3367; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 69.5033 ÷ compras ao S38 1496.3367; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12334,7 +12837,7 @@
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -12343,7 +12846,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4.8565 ÷ compras ao S38 1274.3038; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.7493 ÷ compras ao S38 1274.3038; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12374,7 +12877,7 @@
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -12383,7 +12886,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4.8565 ÷ compras ao S38 1274.3038; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.7493 ÷ compras ao S38 1274.3038; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12917,7 @@
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -12423,7 +12926,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.0867 ÷ compras ao S38 1597.0797; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 8.4589 ÷ compras ao S38 1597.0797; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12454,7 +12957,7 @@
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -12463,7 +12966,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.0867 ÷ compras ao S38 1597.0797; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 8.4589 ÷ compras ao S38 1597.0797; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12494,7 +12997,7 @@
         </is>
       </c>
       <c r="F79" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -12503,7 +13006,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 8.5587 ÷ compras ao S38 2245.7083; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 11.8943 ÷ compras ao S38 2245.7083; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12534,7 +13037,7 @@
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -12543,7 +13046,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 8.5587 ÷ compras ao S38 2245.7083; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 11.8943 ÷ compras ao S38 2245.7083; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12574,7 +13077,7 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -12583,7 +13086,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.4468 ÷ compras ao S38 117.2356; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.6209 ÷ compras ao S38 117.2356; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12614,7 +13117,7 @@
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -12623,7 +13126,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.4468 ÷ compras ao S38 117.2356; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.6209 ÷ compras ao S38 117.2356; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12654,7 +13157,7 @@
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -12663,7 +13166,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.6622 ÷ compras ao S38 436.1311; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2.3100 ÷ compras ao S38 436.1311; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12694,7 +13197,7 @@
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -12703,7 +13206,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.6622 ÷ compras ao S38 436.1311; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 2.3100 ÷ compras ao S38 436.1311; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12734,7 +13237,7 @@
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -12743,7 +13246,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.1830 ÷ compras ao S38 1884.7466; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 9.9825 ÷ compras ao S38 1884.7466; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12774,7 +13277,7 @@
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -12783,7 +13286,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.1830 ÷ compras ao S38 1884.7466; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 9.9825 ÷ compras ao S38 1884.7466; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12814,7 +13317,7 @@
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -12823,7 +13326,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 3.4105 ÷ compras ao S38 894.8737; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4.7397 ÷ compras ao S38 894.8737; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12854,7 +13357,7 @@
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -12863,7 +13366,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 3.4105 ÷ compras ao S38 894.8737; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4.7397 ÷ compras ao S38 894.8737; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12894,7 +13397,7 @@
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -12903,7 +13406,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 8.9121 ÷ compras ao S38 2338.4450; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 12.3855 ÷ compras ao S38 2338.4450; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12934,7 +13437,7 @@
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -12943,7 +13446,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 8.9121 ÷ compras ao S38 2338.4450; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 12.3855 ÷ compras ao S38 2338.4450; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -12974,7 +13477,7 @@
         </is>
       </c>
       <c r="F91" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -12983,7 +13486,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 3.4857 ÷ compras ao S38 914.6124; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4.8442 ÷ compras ao S38 914.6124; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13014,7 +13517,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -13023,7 +13526,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 3.4857 ÷ compras ao S38 914.6124; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4.8442 ÷ compras ao S38 914.6124; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13054,7 +13557,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -13063,7 +13566,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 5.4853 ÷ compras ao S38 1439.2912; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.6232 ÷ compras ao S38 1439.2912; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13094,7 +13597,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -13103,7 +13606,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 5.4853 ÷ compras ao S38 1439.2912; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.6232 ÷ compras ao S38 1439.2912; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13134,7 +13637,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -13143,7 +13646,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.3082 ÷ compras ao S38 343.2676; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.8181 ÷ compras ao S38 343.2676; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13174,7 +13677,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -13183,7 +13686,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.3082 ÷ compras ao S38 343.2676; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.8181 ÷ compras ao S38 343.2676; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13214,7 +13717,7 @@
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -13223,7 +13726,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.1494 ÷ compras ao S38 301.5928; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.5974 ÷ compras ao S38 301.5928; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13254,7 +13757,7 @@
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -13263,7 +13766,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.1494 ÷ compras ao S38 301.5928; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.5974 ÷ compras ao S38 301.5928; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13294,7 +13797,7 @@
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -13303,7 +13806,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.8423 ÷ compras ao S38 221.0197; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.1706 ÷ compras ao S38 221.0197; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13334,7 +13837,7 @@
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -13343,7 +13846,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.8423 ÷ compras ao S38 221.0197; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 1.1706 ÷ compras ao S38 221.0197; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13374,7 +13877,7 @@
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -13383,7 +13886,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 30.5036 ÷ compras ao S38 8003.7958; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 42.3919 ÷ compras ao S38 8003.7958; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13414,7 +13917,7 @@
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -13423,7 +13926,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 30.5036 ÷ compras ao S38 8003.7958; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 42.3919 ÷ compras ao S38 8003.7958; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13454,7 +13957,7 @@
         </is>
       </c>
       <c r="F103" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -13463,7 +13966,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.4347 ÷ compras ao S38 114.0628; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.6041 ÷ compras ao S38 114.0628; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13494,7 +13997,7 @@
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -13503,7 +14006,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.4347 ÷ compras ao S38 114.0628; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 0.6041 ÷ compras ao S38 114.0628; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13534,7 +14037,7 @@
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>0.003617599377013092</v>
+        <v>0.005027507160984955</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -13543,7 +14046,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 20.8237 ÷ compras ao S38 5756.2229; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 28.9395 ÷ compras ao S38 5756.2229; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13574,7 +14077,7 @@
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>0.9963824006229869</v>
+        <v>0.994972492839015</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -13583,7 +14086,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 20.8237 ÷ compras ao S38 5756.2229; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 28.9395 ÷ compras ao S38 5756.2229; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13614,7 +14117,7 @@
         </is>
       </c>
       <c r="F107" s="2" t="n">
-        <v>0.003617599377013093</v>
+        <v>0.005027507160984955</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -13623,7 +14126,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.0718 ÷ compras ao S38 1954.8256; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 9.8279 ÷ compras ao S38 1954.8256; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13654,7 +14157,7 @@
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>0.9963824006229869</v>
+        <v>0.994972492839015</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -13663,7 +14166,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.0718 ÷ compras ao S38 1954.8256; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 9.8279 ÷ compras ao S38 1954.8256; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13694,7 +14197,7 @@
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -13703,7 +14206,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 10.2553 ÷ compras ao S38 2690.8796; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 14.2522 ÷ compras ao S38 2690.8796; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13734,7 +14237,7 @@
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -13743,7 +14246,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 10.2553 ÷ compras ao S38 2690.8796; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 14.2522 ÷ compras ao S38 2690.8796; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13774,7 +14277,7 @@
         </is>
       </c>
       <c r="F111" s="2" t="n">
-        <v>0.003617599377013092</v>
+        <v>0.005027507160984955</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -13783,7 +14286,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4.8669 ÷ compras ao S38 1345.3420; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.7637 ÷ compras ao S38 1345.3420; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13814,7 +14317,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>0.9963824006229869</v>
+        <v>0.994972492839015</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -13823,7 +14326,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 4.8669 ÷ compras ao S38 1345.3420; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.7637 ÷ compras ao S38 1345.3420; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13854,7 +14357,7 @@
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -13863,7 +14366,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.9503 ÷ compras ao S38 1823.6813; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 9.6591 ÷ compras ao S38 1823.6813; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13894,7 +14397,7 @@
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -13903,7 +14406,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 6.9503 ÷ compras ao S38 1823.6813; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 9.6591 ÷ compras ao S38 1823.6813; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13934,7 +14437,7 @@
         </is>
       </c>
       <c r="F115" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267912</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -13943,7 +14446,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 5.0914 ÷ compras ao S38 1335.9168; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.0757 ÷ compras ao S38 1335.9168; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -13974,7 +14477,7 @@
         </is>
       </c>
       <c r="F116" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -13983,7 +14486,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 5.0914 ÷ compras ao S38 1335.9168; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 7.0757 ÷ compras ao S38 1335.9168; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -14014,7 +14517,7 @@
         </is>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0.003811139862305237</v>
+        <v>0.005296477291267913</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -14023,7 +14526,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 12.7106 ÷ compras ao S38 3335.1113; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 17.6643 ÷ compras ao S38 3335.1113; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -14054,7 +14557,7 @@
         </is>
       </c>
       <c r="F118" s="2" t="n">
-        <v>0.9961888601376948</v>
+        <v>0.9947035227087321</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -14063,7 +14566,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 12.7106 ÷ compras ao S38 3335.1113; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
+          <t>BEN 2020 (gás por setor, sem o setor energético) × VBP_GAS_RB, ∝ compras ao S38 dentro de cada setor do BEN (correspondencia_ben_mip_v02.csv); alvo 17.6643 ÷ compras ao S38 3335.1113; HIPÓTESE: mesmo preço por unidade de gás entre compradores; o GAS só vende na própria região; o RAS fecha o VBP do GAS</t>
         </is>
       </c>
     </row>
@@ -20367,7 +20870,7 @@
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>30604.44533452819</v>
+        <v>31637.50993391223</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -20397,7 +20900,7 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>272898.1300593903</v>
+        <v>271865.0654600062</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>

</xml_diff>